<commit_message>
⚡ Actualización manual instantánea de propiedades (con validación estricta de disponibilidad)
</commit_message>
<xml_diff>
--- a/Reporte_Oportunidades_InmoData.xlsx
+++ b/Reporte_Oportunidades_InmoData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,22 +453,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Palermo Hollywood, Palermo</t>
+          <t>Núñez, Capital Federal</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>USD 1.100</t>
+          <t>$ 750.000</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>64 m² tot.2 amb.1 dorm.1 baño1 coch.</t>
+          <t>36 m² tot.1 amb.1 dorm.1 baño</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-dueno-directo-duplex-en-alquiler-palermo-hollywood-53534920.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-dueno-directo-belgrano-nunez-monoambiente-amplio-54157665.html</t>
         </is>
       </c>
     </row>
@@ -480,17 +480,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>$ 600.000</t>
+          <t>USD 1.300</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>50 m² tot.2 amb.1 dorm.1 baño1 coch.</t>
+          <t>67 m² tot.2 amb.1 dorm.1 baño1 coch.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-palermo-alquiler-amoblado-dos-ambientes-frente-59016055.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-alquiler-de-2-ambientes-torres-palermo-view-piso-20-59161431.html</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>$ 449.000</t>
+          <t>$ 550.000</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>23 m² tot.1 amb.1 baño</t>
+          <t>30 m² tot.1 amb.1 baño</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-alquilet-de-mono-ambiente-58432627.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-monoambiente-moderno.-alquiler-temporal.-ideal-para-58420093.html</t>
         </is>
       </c>
     </row>
@@ -524,90 +524,90 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$ 550.000</t>
+          <t>USD 1.300</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>75 m² tot.2 amb.1 dorm.1 baño1 coch.</t>
+          <t>75 m² tot.3 amb.2 dorm.2 baños</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-dos-ambientes-59015930.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-departamento-luminoso-3-ambientes-belgrano-r-59445692.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Palermo, Capital Federal</t>
+          <t>Almagro Norte, Almagro</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$ 670.000</t>
+          <t>$ 480.000</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>75 m² tot.3 amb.2 dorm.2 baños1 coch.</t>
+          <t>33 m² tot.2 amb.1 dorm.1 baño</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-departamento-3-ambientes-59015957.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-dueno-alquila-departamento-de-2-ambientes-en-almagro-59445710.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Palermo Hollywood, Palermo</t>
+          <t>Boedo, Capital Federal</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$ 600.000</t>
+          <t>USD 350</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>50 m² tot.2 amb.1 dorm.1 coch.</t>
+          <t>37 m² tot.1 baño</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-palermo-alquiler-amoblado-2-ambientes-frente-balcon-59015931.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-monoambiente-luminoso-59445685.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Monserrat, Capital Federal</t>
+          <t>Palermo Chico, Palermo</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>$ 980.000</t>
+          <t>$ 700.000</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>95 m² tot.3 amb.2 dorm.1 baño</t>
+          <t>87 m² tot.2 amb.2 dorm.1 baño1 coch.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-amplio-y-luminoso-departamento-al-frente-con-balcon-58197361.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-departamento-en-alquiler-disponible.-59445671.html</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Palermo, Capital Federal</t>
+          <t>Almagro, Capital Federal</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -617,232 +617,232 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>50 m² tot.2 amb.1 dorm.1 baño1 coch.</t>
+          <t>1 m² tot.1 amb.1 baño1 coch.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-palermo-alquiler-amoblado-2-ambientes-disponible-59015873.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-impecable-monoambiente-con-balcon-y-cochera-en-59445596.html</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Recoleta, Capital Federal</t>
+          <t>Flores Norte, Flores</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>USD 2.950</t>
+          <t>$ 799.900</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>145 m² tot.4 amb.3 dorm.2 baños</t>
+          <t>48 m² tot.2 amb.1 dorm.1 baño</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-3-dorm.-recoleta-listo-para-entrar-categoria-59015261.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-2-ambientes-reciclado-a-nuevo-con-balcon-al-frente-59445503.html</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Caballito, Capital Federal</t>
+          <t>Belgrano C, Belgrano</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>$ 600.000</t>
+          <t>$ 1.200.000</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>50 m² tot.2 amb.1 dorm.1 baño1 coch.</t>
+          <t>58 m² tot.2 amb.1 dorm.1 baño</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-alquiler-de-dos-ambientes-ubicado-zona-caballito-59015818.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-alquiler-belgrano-a-estrenar-59445072.html</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Palermo Hollywood, Palermo</t>
+          <t>Belgrano C, Belgrano</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>$ 650.000</t>
+          <t>$ 850.000</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>50 m² tot.2 amb.1 dorm.1 baño1 coch.</t>
+          <t>44 m² tot.1 amb.1 baño</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-palermo-alquiler-amoblado-de-dos-ambientes-frente-59015747.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-excelente-depto.-1-amb-en-belgrano-super-luminoso-y-59432773.html</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Monserrat, Capital Federal</t>
+          <t>Retiro, Capital Federal</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>$ 750.000</t>
+          <t>USD 1.200</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>46 m² tot.2 amb.1 dorm.1 baño</t>
+          <t>55 m² tot.3 amb.2 dorm.1 baño</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-departamento-penthouse-de-2-ambientes-muy-luminoso-y-59015745.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-alquiler-departamento-3-ambientes-dueno-directo-59444889.html</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Lomas de Núñez, Núñez</t>
+          <t>Belgrano, Capital Federal</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>$ 650.000</t>
+          <t>$ 1.800.000</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>35 m² tot.1 amb.1 baño</t>
+          <t>86 m² tot.4 amb.3 dorm.2 baños1 coch.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-hermoso-monoambiente-en-l-59015558.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-semipiso-de-4-amb-frente-balcon-cochera.-piscina-54276180.html</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Almagro Norte, Almagro</t>
+          <t>Belgrano, Capital Federal</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>$ 620.000</t>
+          <t>$ 650.000</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>55 m² tot.2 amb.1 dorm.1 baño</t>
+          <t>41 m² tot.2 amb.1 dorm.1 baño</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-hermoso-2-ambientes-super-luminoso-59015575.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-departamento-2-ambientes-contrafrente-en-belgrano.-59444009.html</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Recoleta, Capital Federal</t>
+          <t>Villa Ortuzar, Capital Federal</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$ 500.000</t>
+          <t>$ 615.000</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>20 m² tot.1 amb.1 dorm.1 baño</t>
+          <t>40 m² tot.2 amb.1 dorm.1 baño</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-alquiler-monoambiente-rod-pena-1500-59015691.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-2-ambientes-luminoso-en-villa-ortuzar-cerca-subte-b-59444037.html</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Almagro Sur, Almagro</t>
+          <t>Lomas de Núñez, Núñez</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$ 900.000</t>
+          <t>$ 725.000</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>60 m² tot.4 amb.3 dorm.1 baño</t>
+          <t>36 m² tot.1 amb.1 baño</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-hermoso-y-funcional-4-amb-en-alquiler-dueno-directo-59013966.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-monoambiente-a-estrenar-en-el-barrio-de-nunez-dueno-59443682.html</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Villa Crespo, Capital Federal</t>
+          <t>Recoleta, Capital Federal</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>$ 1.450.000</t>
+          <t>$ 1.650.000</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>85 m² tot.4 amb.2 dorm.1 baño</t>
+          <t>88 m² tot.2 dorm.2 baños</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-departamento-de-3-ambientes-en-villa-crespo-con-jardin-59014697.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-semipiso-contrafrente-56499422.html</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Barracas, Capital Federal</t>
+          <t>San Nicolás, Capital Federal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>USD 1.400</t>
+          <t>$ 1.200.000</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>130 m² tot.1 amb.1 dorm.1 baño</t>
+          <t>79 m² tot.3 amb.2 dorm.1 baño</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-exclusivo-loft-amoblado-edificio-historico-molina-59015348.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-semipiso-de-categoria:-estilo-clasico-y-confort-59443145.html</t>
         </is>
       </c>
     </row>
@@ -854,171 +854,259 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>$ 500</t>
+          <t>$ 1.000.000</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>65 m² tot.2 amb.2 dorm.1 baño</t>
+          <t>68 m² tot.2 amb.1 dorm.2 baños</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-alquileres-59015436.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-dueno-alquila-2-ambientes-a-estrenar-59443365.html</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Balvanera, Capital Federal</t>
+          <t>Recoleta, Capital Federal</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>$ 900.000</t>
+          <t>$ 550</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>42 m² tot.2 amb.1 dorm.1 baño</t>
+          <t>41 m² tot.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-dueno-directo-alquila-57467613.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-departamento-en-alquiler-ubicado-en-recoleta-59443426.html</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Recoleta, Capital Federal</t>
+          <t>Parque Chas, Capital Federal</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>$ 680.000</t>
+          <t>USD 1.100</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>98 m² tot.2 amb.2 dorm.1 baño1 coch.</t>
+          <t>80 m² tot.3 amb.2 baños</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-departamento-delia-59014982.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-av-de-los-incas-5066-59443328.html</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Palermo, Capital Federal</t>
+          <t>Recoleta, Capital Federal</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>$ 650.000</t>
+          <t>$ 1.899.999</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>50 m² tot.2 amb.1 dorm.1 baño1 coch.</t>
+          <t>54 m² tot.2 amb.1 dorm.2 baños</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-departamento-de-2-ambientes-disponible-zona-palermo-59015015.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-alto-palermo.-2-amb.-2-banos.-opt.-1-coch-cubierta.-53465289.html</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Caballito Sur, Caballito</t>
+          <t>Recoleta, Capital Federal</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>$ 620.000</t>
+          <t>$ 1.400.000</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>35 m² tot.1 amb.1 baño</t>
+          <t>55 m² tot.3 amb.2 dorm.1 baño</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-monoambiente-amplio-apto-prof-dueno-directo-59014866.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-dueno-directo-impecable-3-ambientes-reciclado-en-59443273.html</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Barrio Norte, Capital Federal</t>
+          <t>Caballito Sur, Caballito</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>$ 1.100.000</t>
+          <t>$ 520.000</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>74 m² tot.4 amb.3 dorm.2 baños</t>
+          <t>27 m² tot.1 amb.1 baño</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-dueno-directo-alquila-depto-en-barrio-norte-caba-av-58950544.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-monoambiente-con-balcon-en-caballito-apto-profesional-53473554.html</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Caballito, Capital Federal</t>
+          <t>Recoleta, Capital Federal</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>$ 500</t>
+          <t>$ 1.300.000</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>65 m² tot.2 amb.2 dorm.1 baño</t>
+          <t>62 m² tot.3 amb.2 dorm.1 baño</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-alquileres-59014990.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-alquilo-recoleta-3-ambientes-bano-toilette-terraza-y-59442218.html</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>San Nicolás, Capital Federal</t>
+          <t>Palermo Chico, Palermo</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>$ 900.000</t>
+          <t>$ 1.490.000</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>70 m² tot.2 amb.1 dorm.1 baño</t>
+          <t>83 m² tot.3 amb.3 dorm.1 baño</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-oportunidad-unica-ultimo-piso-terraza-privada-59014251.html</t>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-dueno-directo-alquila-departamento-semipiso-palermo-53550985.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Monserrat, Capital Federal</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>$ 1.100.000</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>75 m² tot.4 amb.2 dorm.1 baño</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-excelente-4-ambientes.-todo-luz.-dueno-directo.-55281756.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Recoleta, Capital Federal</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>$ 850.000</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>48 m² tot.2 amb.1 dorm.1 baño</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-edificio-premium-seg-24-hs-depto-dos-ambientes-59379241.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Palermo, Capital Federal</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>$ 849.999</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>54 m² tot.1 amb.1 dorm.1 baño1 coch.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-botanico-palermo-studio-tipo-loft.-cocina-y-bano-53734134.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Botánico, Palermo</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>USD 1.600</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>140 m² tot.2 amb.2 dorm.1 baño</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.zonaprop.com.ar/propiedades/clasificado/alclappa-vista-panoramica-59442184.html</t>
         </is>
       </c>
     </row>

</xml_diff>